<commit_message>
feat: add webhook notifications and release 1.8.0
Add configurable webhook events, delivery retries, daily summaries, and notification settings for web and Android.

Unify material terminology and import templates across clients, documentation, and tests. Synchronize release versions to 1.8.0.
</commit_message>
<xml_diff>
--- a/tests/fixtures/products.xlsx
+++ b/tests/fixtures/products.xlsx
@@ -13,7 +13,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>商品名称</t>
+          <t>物料名称</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -33,12 +33,12 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>采购价</t>
+          <t>参考采购价</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>销售价</t>
+          <t>参考销售价</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">

</xml_diff>